<commit_message>
docs: add multi-judge lit review to Phase 7.3 report
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/literature-review/phase_7.3/Paper Clusters.xlsx
+++ b/literature-review/phase_7.3/Paper Clusters.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -614,6 +614,21 @@
         <v>2</v>
       </c>
     </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Multi-Judge and Ensemble Evaluation</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Papers on using multiple LLM judges — through majority voting, peer discussion, or consensus methods — to improve reliability and reduce single-model bias in evaluation</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>

</xml_diff>